<commit_message>
Update QA test scripts, results, and screenshots (TC-T-01 to TC-T-13)
- Updated test scripts with improved qa_utils
- Added new test result JSON files (TC-T-12, TC-T-13)
- Updated all screenshots for test cases
- Removed skills folder (cleanup)
- Added backup scripts and parsing utilities
</commit_message>
<xml_diff>
--- a/Quick_TC_list/AIDT 모니터링_운영계_점검 리스트_편집중.xlsx
+++ b/Quick_TC_list/AIDT 모니터링_운영계_점검 리스트_편집중.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\jaehyuk.myung\claude_demo\Demo_13_QA\Quick_TC_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D62D39F2-3055-41A3-8682-D9DD3D0A547A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48466F8F-CB35-4FB4-BC7D-8D1A63191E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37305" yWindow="1785" windowWidth="33015" windowHeight="18375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-35730" yWindow="1695" windowWidth="35370" windowHeight="18375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="개편수정" sheetId="1" r:id="rId1"/>
@@ -456,14 +456,6 @@
   </si>
   <si>
     <t xml:space="preserve"> '좌측 LNB 에서 '교과서' 메뉴 클릭 &gt; 현재창이 전환되며 단원 리스트 노출 &gt; 재구성 하기 &gt; 현재창이 교과서를 재구성하는 화면으로 전환됨 &gt; 임시저장 삭제 버튼이 있다면, 임시저장 삭제 진행&gt; 모달 팝업에서도 삭제 버튼을 눌러서 삭제 진행  &gt; 임시저장 버튼 클릭 &gt; 임시저장 데이터 생성되는지 확인 &gt; 교과서 배포 버튼 클릭 &gt; 모달 팝업에서 확인 버튼 선택 &gt; 모달 팝업 닫히고 토스트 알림이 노출되는지 확인 '배포가 완료 되었습니다.' </t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> '좌측 LNB 에서 '모둠활동' 메뉴 클릭 &gt; 모둠활동 리스트 페이지에서 작성하기 버튼 클릭 &gt; 활동 이름 'sample' 입력 &gt; '타일형' 선택된 상태 &gt; 만들기 버튼 클릭 &gt; 새창으로 sample 이라고 된 창 열리는지 확인</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> '좌측 LNB 에서 '모둠활동' 메뉴 클릭 &gt; 모둠활동 리스트 페이지에서 작성하기 버튼 클릭 &gt; 활동 이름 'sample' 입력 &gt; '모둠형' 선택 &gt; 만들기 버튼 클릭 &gt; 새창으로 sample 이라고 된 창 열리는지 확인</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
@@ -532,12 +524,52 @@
     <t>TC-T-13_group_activity_post_create.py</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> '좌측 LNB 에서 '모둠활동' 메뉴 클릭 &gt; 모둠활동 리스트 페이지에서 작성하기 버튼 클릭 &gt; 활동 이름 'sample' 입력 &gt; '타일형' 선택된 상태 &gt; 만들기 버튼 클릭 &gt; 새창으로 sample 이라고 된 창 열리는지 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>&gt; 열린 창 닫기 &gt; 모둠활동 리스트 페이지에서 'sample' 활동 삭제</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> '좌측 LNB 에서 '모둠활동' 메뉴 클릭 &gt; 모둠활동 리스트 페이지에서 작성하기 버튼 클릭 &gt; 활동 이름 'sample' 입력 &gt; '모둠형' 선택 &gt; 만들기 버튼 클릭 &gt; 새창으로 sample 이라고 된 창 열리는지 확인 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>&gt; 열린 창 닫기 &gt; 모둠활동 리스트 페이지에서 'sample' 활동 삭제</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -636,6 +668,19 @@
     <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Malgun Gothic"/>
       <family val="3"/>
       <charset val="129"/>
@@ -1398,94 +1443,6 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>5334000</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>2219172</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="그림 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B193E534-1CB5-AE52-3AF7-8ED1DD5181BF}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="17164050" y="19154775"/>
-          <a:ext cx="5334000" cy="2219172"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>5495925</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>9794</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="그림 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77EA1F6E-FE9C-8263-6C2C-ABD13639B579}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="17573625" y="21478876"/>
-          <a:ext cx="5495925" cy="2972068"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
@@ -1509,7 +1466,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1553,7 +1510,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1597,7 +1554,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1606,6 +1563,94 @@
         <a:xfrm>
           <a:off x="17573625" y="30984825"/>
           <a:ext cx="6143625" cy="2574065"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>4857751</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>2758869</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="그림 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A132ECA-9ACA-EBD7-CE35-5F1674FF6B65}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17573626" y="19240500"/>
+          <a:ext cx="4857750" cy="2758869"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5410200</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>3046973</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="그림 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{50173955-8C84-3654-6760-59BA82A08401}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17573625" y="22040851"/>
+          <a:ext cx="5410200" cy="3046972"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2172,7 +2217,7 @@
         <v>7</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J17" s="24"/>
       <c r="K17" s="25"/>
@@ -2187,18 +2232,18 @@
         <v>27</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H18" s="24">
         <v>8</v>
       </c>
       <c r="I18" s="24" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J18" s="24"/>
       <c r="K18" s="25"/>
     </row>
-    <row r="19" spans="1:11" ht="176.25" customHeight="1">
+    <row r="19" spans="1:11" ht="220.5" customHeight="1">
       <c r="A19" s="23"/>
       <c r="B19" s="30"/>
       <c r="C19" s="33"/>
@@ -2210,18 +2255,18 @@
         <v>29</v>
       </c>
       <c r="G19" s="21" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="H19" s="24">
         <v>9</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="J19" s="24"/>
       <c r="K19" s="25"/>
     </row>
-    <row r="20" spans="1:11" ht="233.25" customHeight="1">
+    <row r="20" spans="1:11" ht="241.5" customHeight="1">
       <c r="A20" s="23"/>
       <c r="B20" s="30"/>
       <c r="C20" s="33"/>
@@ -2229,13 +2274,13 @@
       <c r="E20" s="53"/>
       <c r="F20" s="55"/>
       <c r="G20" s="21" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="H20" s="24">
         <v>10</v>
       </c>
       <c r="I20" s="24" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J20" s="24"/>
       <c r="K20" s="25"/>
@@ -2247,16 +2292,16 @@
       <c r="D21" s="33"/>
       <c r="E21" s="33"/>
       <c r="F21" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H21" s="24">
         <v>11</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J21" s="24"/>
       <c r="K21" s="25"/>
@@ -2271,13 +2316,13 @@
         <v>30</v>
       </c>
       <c r="G22" s="21" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H22" s="24">
         <v>12</v>
       </c>
       <c r="I22" s="24" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J22" s="24"/>
       <c r="K22" s="25"/>
@@ -2292,13 +2337,13 @@
         <v>31</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H23" s="24">
         <v>13</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J23" s="24"/>
       <c r="K23" s="25"/>

</xml_diff>